<commit_message>
chore(data): update pickLists and riskClassification rules
</commit_message>
<xml_diff>
--- a/data/rules/pickLists.xlsx
+++ b/data/rules/pickLists.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25CA580C-4DD2-4C4F-B81E-25B58C8EABFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47D36F85-5495-4363-BFCC-9159FA8D5A08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2083" uniqueCount="589">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2110" uniqueCount="602">
   <si>
     <t>Path</t>
   </si>
@@ -1787,6 +1787,45 @@
   </si>
   <si>
     <t>Any other attachment type.</t>
+  </si>
+  <si>
+    <t>Tax Evasion</t>
+  </si>
+  <si>
+    <t>Environmental Crime</t>
+  </si>
+  <si>
+    <t>Counterfeiting &amp; Forgery</t>
+  </si>
+  <si>
+    <t>Smuggling</t>
+  </si>
+  <si>
+    <t>Illicit cross-border movement of goods to evade customs duties.</t>
+  </si>
+  <si>
+    <t>Extortion</t>
+  </si>
+  <si>
+    <t>Obtaining money or property through threats or coercion.</t>
+  </si>
+  <si>
+    <t>Illegal Gambling</t>
+  </si>
+  <si>
+    <t>Operating or profiting from unlawful gambling.</t>
+  </si>
+  <si>
+    <t>Kidnapping for Ransom</t>
+  </si>
+  <si>
+    <t>Abduction of persons to extort ransom.</t>
+  </si>
+  <si>
+    <t>Terrorism Financing</t>
+  </si>
+  <si>
+    <t>Funding or material support for terrorism.</t>
   </si>
 </sst>
 </file>
@@ -2193,12 +2232,12 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z1035"/>
+  <dimension ref="A1:Z1043"/>
   <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.54296875" customWidth="1"/>
     <col min="2" max="2" width="26.7265625" customWidth="1"/>
-    <col min="3" max="3" width="19.54296875" customWidth="1"/>
+    <col min="3" max="3" width="21.08984375" customWidth="1"/>
     <col min="5" max="5" width="56.54296875" customWidth="1"/>
     <col min="6" max="6" width="54.08984375" customWidth="1"/>
   </cols>
@@ -9627,145 +9666,151 @@
     </row>
     <row r="648" spans="1:5" ht="29" customHeight="1">
       <c r="A648" s="6" t="s">
-        <v>484</v>
-      </c>
-      <c r="B648" s="6" t="s">
-        <v>485</v>
-      </c>
-      <c r="C648" s="6"/>
-      <c r="D648" s="8"/>
-      <c r="E648" s="6" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="649" spans="1:5" ht="14.5" customHeight="1">
+        <v>472</v>
+      </c>
+      <c r="B648" s="7" t="s">
+        <v>589</v>
+      </c>
+      <c r="C648" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="D648" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E648" s="6"/>
+    </row>
+    <row r="649" spans="1:5" ht="29" customHeight="1">
       <c r="A649" s="6" t="s">
-        <v>484</v>
-      </c>
-      <c r="B649" s="6" t="s">
-        <v>487</v>
-      </c>
-      <c r="C649" s="6"/>
-      <c r="D649" s="8"/>
-      <c r="E649" s="6" t="s">
-        <v>488</v>
-      </c>
+        <v>472</v>
+      </c>
+      <c r="B649" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="C649" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="D649" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E649" s="6"/>
     </row>
     <row r="650" spans="1:5" ht="29" customHeight="1">
       <c r="A650" s="6" t="s">
-        <v>484</v>
-      </c>
-      <c r="B650" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="C650" s="6"/>
-      <c r="D650" s="8"/>
-      <c r="E650" s="6" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="651" spans="1:5" ht="14.5" customHeight="1">
+        <v>472</v>
+      </c>
+      <c r="B650" s="7" t="s">
+        <v>591</v>
+      </c>
+      <c r="C650" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="D650" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="E650" s="6"/>
+    </row>
+    <row r="651" spans="1:5" ht="29" customHeight="1">
       <c r="A651" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="B651" s="6" t="s">
-        <v>491</v>
+      <c r="B651" s="7" t="s">
+        <v>592</v>
       </c>
       <c r="C651" s="6"/>
-      <c r="D651" s="8"/>
+      <c r="D651" s="9"/>
       <c r="E651" s="6" t="s">
-        <v>492</v>
+        <v>593</v>
       </c>
     </row>
     <row r="652" spans="1:5" ht="29" customHeight="1">
       <c r="A652" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="B652" s="6" t="s">
-        <v>493</v>
+      <c r="B652" s="7" t="s">
+        <v>594</v>
       </c>
       <c r="C652" s="6"/>
-      <c r="D652" s="8"/>
+      <c r="D652" s="9"/>
       <c r="E652" s="6" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="653" spans="1:5" ht="14.5" customHeight="1">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="653" spans="1:5" ht="29" customHeight="1">
       <c r="A653" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="B653" s="6" t="s">
-        <v>495</v>
+      <c r="B653" s="7" t="s">
+        <v>596</v>
       </c>
       <c r="C653" s="6"/>
-      <c r="D653" s="8"/>
+      <c r="D653" s="9"/>
       <c r="E653" s="6" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="654" spans="1:5" ht="14.5" customHeight="1">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="654" spans="1:5" ht="29" customHeight="1">
       <c r="A654" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="B654" s="6" t="s">
-        <v>497</v>
+      <c r="B654" s="7" t="s">
+        <v>598</v>
       </c>
       <c r="C654" s="6"/>
-      <c r="D654" s="8"/>
+      <c r="D654" s="9"/>
       <c r="E654" s="6" t="s">
-        <v>498</v>
+        <v>599</v>
       </c>
     </row>
     <row r="655" spans="1:5" ht="29" customHeight="1">
       <c r="A655" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="B655" s="6" t="s">
-        <v>499</v>
+      <c r="B655" s="7" t="s">
+        <v>600</v>
       </c>
       <c r="C655" s="6"/>
-      <c r="D655" s="8"/>
+      <c r="D655" s="9"/>
       <c r="E655" s="6" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="656" spans="1:5" ht="14.5" customHeight="1">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="656" spans="1:5" ht="29" customHeight="1">
       <c r="A656" s="6" t="s">
         <v>484</v>
       </c>
       <c r="B656" s="6" t="s">
-        <v>501</v>
+        <v>485</v>
       </c>
       <c r="C656" s="6"/>
       <c r="D656" s="8"/>
       <c r="E656" s="6" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="657" spans="1:5" ht="29" customHeight="1">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="657" spans="1:5" ht="14.5" customHeight="1">
       <c r="A657" s="6" t="s">
         <v>484</v>
       </c>
       <c r="B657" s="6" t="s">
-        <v>503</v>
+        <v>487</v>
       </c>
       <c r="C657" s="6"/>
       <c r="D657" s="8"/>
       <c r="E657" s="6" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="658" spans="1:5" ht="14.5" customHeight="1">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="658" spans="1:5" ht="29" customHeight="1">
       <c r="A658" s="6" t="s">
         <v>484</v>
       </c>
       <c r="B658" s="6" t="s">
-        <v>505</v>
+        <v>489</v>
       </c>
       <c r="C658" s="6"/>
       <c r="D658" s="8"/>
       <c r="E658" s="6" t="s">
-        <v>506</v>
+        <v>490</v>
       </c>
     </row>
     <row r="659" spans="1:5" ht="14.5" customHeight="1">
@@ -9773,25 +9818,25 @@
         <v>484</v>
       </c>
       <c r="B659" s="6" t="s">
-        <v>507</v>
+        <v>491</v>
       </c>
       <c r="C659" s="6"/>
       <c r="D659" s="8"/>
       <c r="E659" s="6" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="660" spans="1:5" ht="14.5" customHeight="1">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="660" spans="1:5" ht="29" customHeight="1">
       <c r="A660" s="6" t="s">
         <v>484</v>
       </c>
       <c r="B660" s="6" t="s">
-        <v>509</v>
+        <v>493</v>
       </c>
       <c r="C660" s="6"/>
       <c r="D660" s="8"/>
       <c r="E660" s="6" t="s">
-        <v>510</v>
+        <v>494</v>
       </c>
     </row>
     <row r="661" spans="1:5" ht="14.5" customHeight="1">
@@ -9799,12 +9844,12 @@
         <v>484</v>
       </c>
       <c r="B661" s="6" t="s">
-        <v>511</v>
+        <v>495</v>
       </c>
       <c r="C661" s="6"/>
       <c r="D661" s="8"/>
       <c r="E661" s="6" t="s">
-        <v>512</v>
+        <v>496</v>
       </c>
     </row>
     <row r="662" spans="1:5" ht="14.5" customHeight="1">
@@ -9812,116 +9857,116 @@
         <v>484</v>
       </c>
       <c r="B662" s="6" t="s">
-        <v>30</v>
+        <v>497</v>
       </c>
       <c r="C662" s="6"/>
       <c r="D662" s="8"/>
       <c r="E662" s="6" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="663" spans="1:5" ht="14.5" customHeight="1">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="663" spans="1:5" ht="29" customHeight="1">
       <c r="A663" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B663" s="6" t="s">
-        <v>515</v>
+        <v>499</v>
       </c>
       <c r="C663" s="6"/>
       <c r="D663" s="8"/>
       <c r="E663" s="6" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="664" spans="1:5" ht="29" customHeight="1">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="664" spans="1:5" ht="14.5" customHeight="1">
       <c r="A664" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B664" s="6" t="s">
-        <v>93</v>
+        <v>501</v>
       </c>
       <c r="C664" s="6"/>
       <c r="D664" s="8"/>
       <c r="E664" s="6" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="665" spans="1:5" ht="14.5" customHeight="1">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="665" spans="1:5" ht="29" customHeight="1">
       <c r="A665" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B665" s="6" t="s">
-        <v>518</v>
+        <v>503</v>
       </c>
       <c r="C665" s="6"/>
       <c r="D665" s="8"/>
       <c r="E665" s="6" t="s">
-        <v>519</v>
+        <v>504</v>
       </c>
     </row>
     <row r="666" spans="1:5" ht="14.5" customHeight="1">
       <c r="A666" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B666" s="6" t="s">
-        <v>520</v>
+        <v>505</v>
       </c>
       <c r="C666" s="6"/>
       <c r="D666" s="8"/>
       <c r="E666" s="6" t="s">
-        <v>521</v>
+        <v>506</v>
       </c>
     </row>
     <row r="667" spans="1:5" ht="14.5" customHeight="1">
       <c r="A667" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B667" s="6" t="s">
-        <v>522</v>
+        <v>507</v>
       </c>
       <c r="C667" s="6"/>
       <c r="D667" s="8"/>
       <c r="E667" s="6" t="s">
-        <v>523</v>
+        <v>508</v>
       </c>
     </row>
     <row r="668" spans="1:5" ht="14.5" customHeight="1">
       <c r="A668" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B668" s="6" t="s">
-        <v>524</v>
+        <v>509</v>
       </c>
       <c r="C668" s="6"/>
       <c r="D668" s="8"/>
       <c r="E668" s="6" t="s">
-        <v>525</v>
+        <v>510</v>
       </c>
     </row>
     <row r="669" spans="1:5" ht="14.5" customHeight="1">
       <c r="A669" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B669" s="6" t="s">
-        <v>526</v>
+        <v>511</v>
       </c>
       <c r="C669" s="6"/>
       <c r="D669" s="8"/>
       <c r="E669" s="6" t="s">
-        <v>527</v>
+        <v>512</v>
       </c>
     </row>
     <row r="670" spans="1:5" ht="14.5" customHeight="1">
       <c r="A670" s="6" t="s">
-        <v>514</v>
+        <v>484</v>
       </c>
       <c r="B670" s="6" t="s">
-        <v>101</v>
+        <v>30</v>
       </c>
       <c r="C670" s="6"/>
       <c r="D670" s="8"/>
       <c r="E670" s="6" t="s">
-        <v>528</v>
+        <v>513</v>
       </c>
     </row>
     <row r="671" spans="1:5" ht="14.5" customHeight="1">
@@ -9929,25 +9974,25 @@
         <v>514</v>
       </c>
       <c r="B671" s="6" t="s">
-        <v>529</v>
+        <v>515</v>
       </c>
       <c r="C671" s="6"/>
       <c r="D671" s="8"/>
       <c r="E671" s="6" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="672" spans="1:5" ht="14.5" customHeight="1">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="672" spans="1:5" ht="29" customHeight="1">
       <c r="A672" s="6" t="s">
         <v>514</v>
       </c>
       <c r="B672" s="6" t="s">
-        <v>531</v>
+        <v>93</v>
       </c>
       <c r="C672" s="6"/>
       <c r="D672" s="8"/>
       <c r="E672" s="6" t="s">
-        <v>532</v>
+        <v>517</v>
       </c>
     </row>
     <row r="673" spans="1:5" ht="14.5" customHeight="1">
@@ -9955,12 +10000,12 @@
         <v>514</v>
       </c>
       <c r="B673" s="6" t="s">
-        <v>533</v>
+        <v>518</v>
       </c>
       <c r="C673" s="6"/>
       <c r="D673" s="8"/>
       <c r="E673" s="6" t="s">
-        <v>534</v>
+        <v>519</v>
       </c>
     </row>
     <row r="674" spans="1:5" ht="14.5" customHeight="1">
@@ -9968,12 +10013,12 @@
         <v>514</v>
       </c>
       <c r="B674" s="6" t="s">
-        <v>97</v>
+        <v>520</v>
       </c>
       <c r="C674" s="6"/>
       <c r="D674" s="8"/>
       <c r="E674" s="6" t="s">
-        <v>535</v>
+        <v>521</v>
       </c>
     </row>
     <row r="675" spans="1:5" ht="14.5" customHeight="1">
@@ -9981,12 +10026,12 @@
         <v>514</v>
       </c>
       <c r="B675" s="6" t="s">
-        <v>536</v>
+        <v>522</v>
       </c>
       <c r="C675" s="6"/>
       <c r="D675" s="8"/>
       <c r="E675" s="6" t="s">
-        <v>537</v>
+        <v>523</v>
       </c>
     </row>
     <row r="676" spans="1:5" ht="14.5" customHeight="1">
@@ -9994,12 +10039,12 @@
         <v>514</v>
       </c>
       <c r="B676" s="6" t="s">
-        <v>538</v>
+        <v>524</v>
       </c>
       <c r="C676" s="6"/>
       <c r="D676" s="8"/>
       <c r="E676" s="6" t="s">
-        <v>539</v>
+        <v>525</v>
       </c>
     </row>
     <row r="677" spans="1:5" ht="14.5" customHeight="1">
@@ -10007,25 +10052,25 @@
         <v>514</v>
       </c>
       <c r="B677" s="6" t="s">
-        <v>540</v>
+        <v>526</v>
       </c>
       <c r="C677" s="6"/>
       <c r="D677" s="8"/>
       <c r="E677" s="6" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="678" spans="1:5" ht="29" customHeight="1">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="678" spans="1:5" ht="14.5" customHeight="1">
       <c r="A678" s="6" t="s">
         <v>514</v>
       </c>
       <c r="B678" s="6" t="s">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="C678" s="6"/>
       <c r="D678" s="8"/>
       <c r="E678" s="6" t="s">
-        <v>542</v>
+        <v>528</v>
       </c>
     </row>
     <row r="679" spans="1:5" ht="14.5" customHeight="1">
@@ -10033,168 +10078,168 @@
         <v>514</v>
       </c>
       <c r="B679" s="6" t="s">
-        <v>30</v>
+        <v>529</v>
       </c>
       <c r="C679" s="6"/>
       <c r="D679" s="8"/>
       <c r="E679" s="6" t="s">
-        <v>543</v>
+        <v>530</v>
       </c>
     </row>
     <row r="680" spans="1:5" ht="14.5" customHeight="1">
       <c r="A680" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="B680" s="7" t="s">
-        <v>545</v>
+        <v>514</v>
+      </c>
+      <c r="B680" s="6" t="s">
+        <v>531</v>
       </c>
       <c r="C680" s="6"/>
       <c r="D680" s="8"/>
-      <c r="E680" s="7" t="s">
-        <v>546</v>
+      <c r="E680" s="6" t="s">
+        <v>532</v>
       </c>
     </row>
     <row r="681" spans="1:5" ht="14.5" customHeight="1">
       <c r="A681" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="B681" s="7" t="s">
-        <v>547</v>
+        <v>514</v>
+      </c>
+      <c r="B681" s="6" t="s">
+        <v>533</v>
       </c>
       <c r="C681" s="6"/>
       <c r="D681" s="8"/>
-      <c r="E681" s="7" t="s">
-        <v>548</v>
+      <c r="E681" s="6" t="s">
+        <v>534</v>
       </c>
     </row>
     <row r="682" spans="1:5" ht="14.5" customHeight="1">
       <c r="A682" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="B682" s="7" t="s">
-        <v>549</v>
+        <v>514</v>
+      </c>
+      <c r="B682" s="6" t="s">
+        <v>97</v>
       </c>
       <c r="C682" s="6"/>
       <c r="D682" s="8"/>
-      <c r="E682" s="7" t="s">
-        <v>550</v>
+      <c r="E682" s="6" t="s">
+        <v>535</v>
       </c>
     </row>
     <row r="683" spans="1:5" ht="14.5" customHeight="1">
       <c r="A683" s="6" t="s">
-        <v>544</v>
-      </c>
-      <c r="B683" s="7" t="s">
-        <v>551</v>
+        <v>514</v>
+      </c>
+      <c r="B683" s="6" t="s">
+        <v>536</v>
       </c>
       <c r="C683" s="6"/>
       <c r="D683" s="8"/>
-      <c r="E683" s="7" t="s">
-        <v>552</v>
+      <c r="E683" s="6" t="s">
+        <v>537</v>
       </c>
     </row>
     <row r="684" spans="1:5" ht="14.5" customHeight="1">
       <c r="A684" s="6" t="s">
-        <v>553</v>
+        <v>514</v>
       </c>
       <c r="B684" s="6" t="s">
-        <v>554</v>
+        <v>538</v>
       </c>
       <c r="C684" s="6"/>
       <c r="D684" s="8"/>
       <c r="E684" s="6" t="s">
-        <v>555</v>
+        <v>539</v>
       </c>
     </row>
     <row r="685" spans="1:5" ht="14.5" customHeight="1">
       <c r="A685" s="6" t="s">
-        <v>553</v>
+        <v>514</v>
       </c>
       <c r="B685" s="6" t="s">
-        <v>556</v>
+        <v>540</v>
       </c>
       <c r="C685" s="6"/>
       <c r="D685" s="8"/>
       <c r="E685" s="6" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="686" spans="1:5" ht="14.5" customHeight="1">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="686" spans="1:5" ht="29" customHeight="1">
       <c r="A686" s="6" t="s">
-        <v>553</v>
+        <v>514</v>
       </c>
       <c r="B686" s="6" t="s">
-        <v>558</v>
+        <v>80</v>
       </c>
       <c r="C686" s="6"/>
       <c r="D686" s="8"/>
       <c r="E686" s="6" t="s">
-        <v>559</v>
+        <v>542</v>
       </c>
     </row>
     <row r="687" spans="1:5" ht="14.5" customHeight="1">
       <c r="A687" s="6" t="s">
-        <v>553</v>
+        <v>514</v>
       </c>
       <c r="B687" s="6" t="s">
-        <v>560</v>
+        <v>30</v>
       </c>
       <c r="C687" s="6"/>
       <c r="D687" s="8"/>
       <c r="E687" s="6" t="s">
-        <v>561</v>
+        <v>543</v>
       </c>
     </row>
     <row r="688" spans="1:5" ht="14.5" customHeight="1">
       <c r="A688" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="B688" s="6" t="s">
-        <v>562</v>
+        <v>544</v>
+      </c>
+      <c r="B688" s="7" t="s">
+        <v>545</v>
       </c>
       <c r="C688" s="6"/>
       <c r="D688" s="8"/>
-      <c r="E688" s="6" t="s">
-        <v>563</v>
+      <c r="E688" s="7" t="s">
+        <v>546</v>
       </c>
     </row>
     <row r="689" spans="1:5" ht="14.5" customHeight="1">
       <c r="A689" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="B689" s="6" t="s">
-        <v>564</v>
+        <v>544</v>
+      </c>
+      <c r="B689" s="7" t="s">
+        <v>547</v>
       </c>
       <c r="C689" s="6"/>
       <c r="D689" s="8"/>
-      <c r="E689" s="6" t="s">
-        <v>565</v>
+      <c r="E689" s="7" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="690" spans="1:5" ht="14.5" customHeight="1">
       <c r="A690" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="B690" s="6" t="s">
-        <v>566</v>
+        <v>544</v>
+      </c>
+      <c r="B690" s="7" t="s">
+        <v>549</v>
       </c>
       <c r="C690" s="6"/>
       <c r="D690" s="8"/>
-      <c r="E690" s="6" t="s">
-        <v>567</v>
+      <c r="E690" s="7" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="691" spans="1:5" ht="14.5" customHeight="1">
       <c r="A691" s="6" t="s">
-        <v>553</v>
-      </c>
-      <c r="B691" s="6" t="s">
-        <v>568</v>
+        <v>544</v>
+      </c>
+      <c r="B691" s="7" t="s">
+        <v>551</v>
       </c>
       <c r="C691" s="6"/>
       <c r="D691" s="8"/>
-      <c r="E691" s="6" t="s">
-        <v>569</v>
+      <c r="E691" s="7" t="s">
+        <v>552</v>
       </c>
     </row>
     <row r="692" spans="1:5" ht="14.5" customHeight="1">
@@ -10202,12 +10247,12 @@
         <v>553</v>
       </c>
       <c r="B692" s="6" t="s">
-        <v>570</v>
+        <v>554</v>
       </c>
       <c r="C692" s="6"/>
       <c r="D692" s="8"/>
       <c r="E692" s="6" t="s">
-        <v>571</v>
+        <v>555</v>
       </c>
     </row>
     <row r="693" spans="1:5" ht="14.5" customHeight="1">
@@ -10215,12 +10260,12 @@
         <v>553</v>
       </c>
       <c r="B693" s="6" t="s">
-        <v>572</v>
+        <v>556</v>
       </c>
       <c r="C693" s="6"/>
       <c r="D693" s="8"/>
       <c r="E693" s="6" t="s">
-        <v>573</v>
+        <v>557</v>
       </c>
     </row>
     <row r="694" spans="1:5" ht="14.5" customHeight="1">
@@ -10228,12 +10273,12 @@
         <v>553</v>
       </c>
       <c r="B694" s="6" t="s">
-        <v>574</v>
+        <v>558</v>
       </c>
       <c r="C694" s="6"/>
       <c r="D694" s="8"/>
       <c r="E694" s="6" t="s">
-        <v>575</v>
+        <v>559</v>
       </c>
     </row>
     <row r="695" spans="1:5" ht="14.5" customHeight="1">
@@ -10241,12 +10286,12 @@
         <v>553</v>
       </c>
       <c r="B695" s="6" t="s">
-        <v>576</v>
+        <v>560</v>
       </c>
       <c r="C695" s="6"/>
       <c r="D695" s="8"/>
       <c r="E695" s="6" t="s">
-        <v>577</v>
+        <v>561</v>
       </c>
     </row>
     <row r="696" spans="1:5" ht="14.5" customHeight="1">
@@ -10254,108 +10299,124 @@
         <v>553</v>
       </c>
       <c r="B696" s="6" t="s">
-        <v>30</v>
+        <v>562</v>
       </c>
       <c r="C696" s="6"/>
       <c r="D696" s="8"/>
       <c r="E696" s="6" t="s">
-        <v>578</v>
+        <v>563</v>
       </c>
     </row>
     <row r="697" spans="1:5" ht="14.5" customHeight="1">
       <c r="A697" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B697" s="11" t="s">
-        <v>117</v>
+        <v>553</v>
+      </c>
+      <c r="B697" s="6" t="s">
+        <v>564</v>
       </c>
       <c r="C697" s="6"/>
       <c r="D697" s="8"/>
-      <c r="E697" s="6"/>
+      <c r="E697" s="6" t="s">
+        <v>565</v>
+      </c>
     </row>
     <row r="698" spans="1:5" ht="14.5" customHeight="1">
       <c r="A698" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B698" s="11" t="s">
-        <v>118</v>
+        <v>553</v>
+      </c>
+      <c r="B698" s="6" t="s">
+        <v>566</v>
       </c>
       <c r="C698" s="6"/>
       <c r="D698" s="8"/>
-      <c r="E698" s="6"/>
+      <c r="E698" s="6" t="s">
+        <v>567</v>
+      </c>
     </row>
     <row r="699" spans="1:5" ht="14.5" customHeight="1">
       <c r="A699" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B699" s="11" t="s">
-        <v>119</v>
+        <v>553</v>
+      </c>
+      <c r="B699" s="6" t="s">
+        <v>568</v>
       </c>
       <c r="C699" s="6"/>
       <c r="D699" s="8"/>
-      <c r="E699" s="6"/>
+      <c r="E699" s="6" t="s">
+        <v>569</v>
+      </c>
     </row>
     <row r="700" spans="1:5" ht="14.5" customHeight="1">
       <c r="A700" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B700" s="11" t="s">
-        <v>120</v>
+        <v>553</v>
+      </c>
+      <c r="B700" s="6" t="s">
+        <v>570</v>
       </c>
       <c r="C700" s="6"/>
       <c r="D700" s="8"/>
-      <c r="E700" s="6"/>
+      <c r="E700" s="6" t="s">
+        <v>571</v>
+      </c>
     </row>
     <row r="701" spans="1:5" ht="14.5" customHeight="1">
       <c r="A701" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B701" s="11" t="s">
-        <v>121</v>
+        <v>553</v>
+      </c>
+      <c r="B701" s="6" t="s">
+        <v>572</v>
       </c>
       <c r="C701" s="6"/>
       <c r="D701" s="8"/>
-      <c r="E701" s="6"/>
+      <c r="E701" s="6" t="s">
+        <v>573</v>
+      </c>
     </row>
     <row r="702" spans="1:5" ht="14.5" customHeight="1">
       <c r="A702" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B702" s="11" t="s">
-        <v>122</v>
+        <v>553</v>
+      </c>
+      <c r="B702" s="6" t="s">
+        <v>574</v>
       </c>
       <c r="C702" s="6"/>
       <c r="D702" s="8"/>
-      <c r="E702" s="6"/>
+      <c r="E702" s="6" t="s">
+        <v>575</v>
+      </c>
     </row>
     <row r="703" spans="1:5" ht="14.5" customHeight="1">
       <c r="A703" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B703" s="11" t="s">
-        <v>123</v>
+        <v>553</v>
+      </c>
+      <c r="B703" s="6" t="s">
+        <v>576</v>
       </c>
       <c r="C703" s="6"/>
       <c r="D703" s="8"/>
-      <c r="E703" s="6"/>
+      <c r="E703" s="6" t="s">
+        <v>577</v>
+      </c>
     </row>
     <row r="704" spans="1:5" ht="14.5" customHeight="1">
       <c r="A704" s="6" t="s">
-        <v>579</v>
-      </c>
-      <c r="B704" s="11" t="s">
-        <v>124</v>
+        <v>553</v>
+      </c>
+      <c r="B704" s="6" t="s">
+        <v>30</v>
       </c>
       <c r="C704" s="6"/>
       <c r="D704" s="8"/>
-      <c r="E704" s="6"/>
+      <c r="E704" s="6" t="s">
+        <v>578</v>
+      </c>
     </row>
     <row r="705" spans="1:5" ht="14.5" customHeight="1">
       <c r="A705" s="6" t="s">
         <v>579</v>
       </c>
       <c r="B705" s="11" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="C705" s="6"/>
       <c r="D705" s="8"/>
@@ -10366,7 +10427,7 @@
         <v>579</v>
       </c>
       <c r="B706" s="11" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="C706" s="6"/>
       <c r="D706" s="8"/>
@@ -10377,7 +10438,7 @@
         <v>579</v>
       </c>
       <c r="B707" s="11" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="C707" s="6"/>
       <c r="D707" s="8"/>
@@ -10388,7 +10449,7 @@
         <v>579</v>
       </c>
       <c r="B708" s="11" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="C708" s="6"/>
       <c r="D708" s="8"/>
@@ -10399,7 +10460,7 @@
         <v>579</v>
       </c>
       <c r="B709" s="11" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="C709" s="6"/>
       <c r="D709" s="8"/>
@@ -10410,7 +10471,7 @@
         <v>579</v>
       </c>
       <c r="B710" s="11" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="C710" s="6"/>
       <c r="D710" s="8"/>
@@ -10421,7 +10482,7 @@
         <v>579</v>
       </c>
       <c r="B711" s="11" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="C711" s="6"/>
       <c r="D711" s="8"/>
@@ -10432,7 +10493,7 @@
         <v>579</v>
       </c>
       <c r="B712" s="11" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C712" s="6"/>
       <c r="D712" s="8"/>
@@ -10443,7 +10504,7 @@
         <v>579</v>
       </c>
       <c r="B713" s="11" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="C713" s="6"/>
       <c r="D713" s="8"/>
@@ -10454,7 +10515,7 @@
         <v>579</v>
       </c>
       <c r="B714" s="11" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="C714" s="6"/>
       <c r="D714" s="8"/>
@@ -10465,7 +10526,7 @@
         <v>579</v>
       </c>
       <c r="B715" s="11" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="C715" s="6"/>
       <c r="D715" s="8"/>
@@ -10476,7 +10537,7 @@
         <v>579</v>
       </c>
       <c r="B716" s="11" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="C716" s="6"/>
       <c r="D716" s="8"/>
@@ -10487,7 +10548,7 @@
         <v>579</v>
       </c>
       <c r="B717" s="11" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="C717" s="6"/>
       <c r="D717" s="8"/>
@@ -10498,7 +10559,7 @@
         <v>579</v>
       </c>
       <c r="B718" s="11" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C718" s="6"/>
       <c r="D718" s="8"/>
@@ -10509,7 +10570,7 @@
         <v>579</v>
       </c>
       <c r="B719" s="11" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C719" s="6"/>
       <c r="D719" s="8"/>
@@ -10520,7 +10581,7 @@
         <v>579</v>
       </c>
       <c r="B720" s="11" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C720" s="6"/>
       <c r="D720" s="8"/>
@@ -10531,7 +10592,7 @@
         <v>579</v>
       </c>
       <c r="B721" s="11" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="C721" s="6"/>
       <c r="D721" s="8"/>
@@ -10542,7 +10603,7 @@
         <v>579</v>
       </c>
       <c r="B722" s="11" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C722" s="6"/>
       <c r="D722" s="8"/>
@@ -10553,7 +10614,7 @@
         <v>579</v>
       </c>
       <c r="B723" s="11" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C723" s="6"/>
       <c r="D723" s="8"/>
@@ -10564,7 +10625,7 @@
         <v>579</v>
       </c>
       <c r="B724" s="11" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C724" s="6"/>
       <c r="D724" s="8"/>
@@ -10575,7 +10636,7 @@
         <v>579</v>
       </c>
       <c r="B725" s="11" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C725" s="6"/>
       <c r="D725" s="8"/>
@@ -10586,7 +10647,7 @@
         <v>579</v>
       </c>
       <c r="B726" s="11" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C726" s="6"/>
       <c r="D726" s="8"/>
@@ -10597,7 +10658,7 @@
         <v>579</v>
       </c>
       <c r="B727" s="11" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C727" s="6"/>
       <c r="D727" s="8"/>
@@ -10608,7 +10669,7 @@
         <v>579</v>
       </c>
       <c r="B728" s="11" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C728" s="6"/>
       <c r="D728" s="8"/>
@@ -10619,7 +10680,7 @@
         <v>579</v>
       </c>
       <c r="B729" s="11" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C729" s="6"/>
       <c r="D729" s="8"/>
@@ -10630,7 +10691,7 @@
         <v>579</v>
       </c>
       <c r="B730" s="11" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C730" s="6"/>
       <c r="D730" s="8"/>
@@ -10641,7 +10702,7 @@
         <v>579</v>
       </c>
       <c r="B731" s="11" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C731" s="6"/>
       <c r="D731" s="8"/>
@@ -10652,7 +10713,7 @@
         <v>579</v>
       </c>
       <c r="B732" s="11" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C732" s="6"/>
       <c r="D732" s="8"/>
@@ -10663,7 +10724,7 @@
         <v>579</v>
       </c>
       <c r="B733" s="11" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="C733" s="6"/>
       <c r="D733" s="8"/>
@@ -10674,7 +10735,7 @@
         <v>579</v>
       </c>
       <c r="B734" s="11" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C734" s="6"/>
       <c r="D734" s="8"/>
@@ -10685,7 +10746,7 @@
         <v>579</v>
       </c>
       <c r="B735" s="11" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C735" s="6"/>
       <c r="D735" s="8"/>
@@ -10696,7 +10757,7 @@
         <v>579</v>
       </c>
       <c r="B736" s="11" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C736" s="6"/>
       <c r="D736" s="8"/>
@@ -10707,7 +10768,7 @@
         <v>579</v>
       </c>
       <c r="B737" s="11" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C737" s="6"/>
       <c r="D737" s="8"/>
@@ -10718,7 +10779,7 @@
         <v>579</v>
       </c>
       <c r="B738" s="11" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="C738" s="6"/>
       <c r="D738" s="8"/>
@@ -10729,7 +10790,7 @@
         <v>579</v>
       </c>
       <c r="B739" s="11" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="C739" s="6"/>
       <c r="D739" s="8"/>
@@ -10740,7 +10801,7 @@
         <v>579</v>
       </c>
       <c r="B740" s="11" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C740" s="6"/>
       <c r="D740" s="8"/>
@@ -10751,7 +10812,7 @@
         <v>579</v>
       </c>
       <c r="B741" s="11" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="C741" s="6"/>
       <c r="D741" s="8"/>
@@ -10762,7 +10823,7 @@
         <v>579</v>
       </c>
       <c r="B742" s="11" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C742" s="6"/>
       <c r="D742" s="8"/>
@@ -10773,7 +10834,7 @@
         <v>579</v>
       </c>
       <c r="B743" s="11" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="C743" s="6"/>
       <c r="D743" s="8"/>
@@ -10784,7 +10845,7 @@
         <v>579</v>
       </c>
       <c r="B744" s="11" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="C744" s="6"/>
       <c r="D744" s="8"/>
@@ -10795,7 +10856,7 @@
         <v>579</v>
       </c>
       <c r="B745" s="11" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="C745" s="6"/>
       <c r="D745" s="8"/>
@@ -10806,7 +10867,7 @@
         <v>579</v>
       </c>
       <c r="B746" s="11" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="C746" s="6"/>
       <c r="D746" s="8"/>
@@ -10817,7 +10878,7 @@
         <v>579</v>
       </c>
       <c r="B747" s="11" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C747" s="6"/>
       <c r="D747" s="8"/>
@@ -10828,7 +10889,7 @@
         <v>579</v>
       </c>
       <c r="B748" s="11" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="C748" s="6"/>
       <c r="D748" s="8"/>
@@ -10839,7 +10900,7 @@
         <v>579</v>
       </c>
       <c r="B749" s="11" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="C749" s="6"/>
       <c r="D749" s="8"/>
@@ -10850,7 +10911,7 @@
         <v>579</v>
       </c>
       <c r="B750" s="11" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="C750" s="6"/>
       <c r="D750" s="8"/>
@@ -10861,7 +10922,7 @@
         <v>579</v>
       </c>
       <c r="B751" s="11" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="C751" s="6"/>
       <c r="D751" s="8"/>
@@ -10872,7 +10933,7 @@
         <v>579</v>
       </c>
       <c r="B752" s="11" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C752" s="6"/>
       <c r="D752" s="8"/>
@@ -10883,7 +10944,7 @@
         <v>579</v>
       </c>
       <c r="B753" s="11" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="C753" s="6"/>
       <c r="D753" s="8"/>
@@ -10894,7 +10955,7 @@
         <v>579</v>
       </c>
       <c r="B754" s="11" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C754" s="6"/>
       <c r="D754" s="8"/>
@@ -10905,7 +10966,7 @@
         <v>579</v>
       </c>
       <c r="B755" s="11" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C755" s="6"/>
       <c r="D755" s="8"/>
@@ -10916,7 +10977,7 @@
         <v>579</v>
       </c>
       <c r="B756" s="11" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="C756" s="6"/>
       <c r="D756" s="8"/>
@@ -10927,7 +10988,7 @@
         <v>579</v>
       </c>
       <c r="B757" s="11" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C757" s="6"/>
       <c r="D757" s="8"/>
@@ -10938,7 +10999,7 @@
         <v>579</v>
       </c>
       <c r="B758" s="11" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C758" s="6"/>
       <c r="D758" s="8"/>
@@ -10949,7 +11010,7 @@
         <v>579</v>
       </c>
       <c r="B759" s="11" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C759" s="6"/>
       <c r="D759" s="8"/>
@@ -10960,7 +11021,7 @@
         <v>579</v>
       </c>
       <c r="B760" s="11" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C760" s="6"/>
       <c r="D760" s="8"/>
@@ -10971,7 +11032,7 @@
         <v>579</v>
       </c>
       <c r="B761" s="11" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C761" s="6"/>
       <c r="D761" s="8"/>
@@ -10982,7 +11043,7 @@
         <v>579</v>
       </c>
       <c r="B762" s="11" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C762" s="6"/>
       <c r="D762" s="8"/>
@@ -10993,7 +11054,7 @@
         <v>579</v>
       </c>
       <c r="B763" s="11" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="C763" s="6"/>
       <c r="D763" s="8"/>
@@ -11004,7 +11065,7 @@
         <v>579</v>
       </c>
       <c r="B764" s="11" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="C764" s="6"/>
       <c r="D764" s="8"/>
@@ -11015,7 +11076,7 @@
         <v>579</v>
       </c>
       <c r="B765" s="11" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C765" s="6"/>
       <c r="D765" s="8"/>
@@ -11026,7 +11087,7 @@
         <v>579</v>
       </c>
       <c r="B766" s="11" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="C766" s="6"/>
       <c r="D766" s="8"/>
@@ -11037,7 +11098,7 @@
         <v>579</v>
       </c>
       <c r="B767" s="11" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="C767" s="6"/>
       <c r="D767" s="8"/>
@@ -11048,7 +11109,7 @@
         <v>579</v>
       </c>
       <c r="B768" s="11" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C768" s="6"/>
       <c r="D768" s="8"/>
@@ -11059,7 +11120,7 @@
         <v>579</v>
       </c>
       <c r="B769" s="11" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="C769" s="6"/>
       <c r="D769" s="8"/>
@@ -11070,7 +11131,7 @@
         <v>579</v>
       </c>
       <c r="B770" s="11" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="C770" s="6"/>
       <c r="D770" s="8"/>
@@ -11081,7 +11142,7 @@
         <v>579</v>
       </c>
       <c r="B771" s="11" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C771" s="6"/>
       <c r="D771" s="8"/>
@@ -11092,7 +11153,7 @@
         <v>579</v>
       </c>
       <c r="B772" s="11" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="C772" s="6"/>
       <c r="D772" s="8"/>
@@ -11103,7 +11164,7 @@
         <v>579</v>
       </c>
       <c r="B773" s="11" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="C773" s="6"/>
       <c r="D773" s="8"/>
@@ -11114,7 +11175,7 @@
         <v>579</v>
       </c>
       <c r="B774" s="11" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="C774" s="6"/>
       <c r="D774" s="8"/>
@@ -11125,7 +11186,7 @@
         <v>579</v>
       </c>
       <c r="B775" s="11" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C775" s="6"/>
       <c r="D775" s="8"/>
@@ -11136,7 +11197,7 @@
         <v>579</v>
       </c>
       <c r="B776" s="11" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="C776" s="6"/>
       <c r="D776" s="8"/>
@@ -11147,7 +11208,7 @@
         <v>579</v>
       </c>
       <c r="B777" s="11" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="C777" s="6"/>
       <c r="D777" s="8"/>
@@ -11158,7 +11219,7 @@
         <v>579</v>
       </c>
       <c r="B778" s="11" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C778" s="6"/>
       <c r="D778" s="8"/>
@@ -11169,7 +11230,7 @@
         <v>579</v>
       </c>
       <c r="B779" s="11" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="C779" s="6"/>
       <c r="D779" s="8"/>
@@ -11180,7 +11241,7 @@
         <v>579</v>
       </c>
       <c r="B780" s="11" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="C780" s="6"/>
       <c r="D780" s="8"/>
@@ -11191,7 +11252,7 @@
         <v>579</v>
       </c>
       <c r="B781" s="11" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="C781" s="6"/>
       <c r="D781" s="8"/>
@@ -11202,7 +11263,7 @@
         <v>579</v>
       </c>
       <c r="B782" s="11" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="C782" s="6"/>
       <c r="D782" s="8"/>
@@ -11213,7 +11274,7 @@
         <v>579</v>
       </c>
       <c r="B783" s="11" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="C783" s="6"/>
       <c r="D783" s="8"/>
@@ -11224,7 +11285,7 @@
         <v>579</v>
       </c>
       <c r="B784" s="11" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="C784" s="6"/>
       <c r="D784" s="8"/>
@@ -11235,7 +11296,7 @@
         <v>579</v>
       </c>
       <c r="B785" s="11" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C785" s="6"/>
       <c r="D785" s="8"/>
@@ -11246,7 +11307,7 @@
         <v>579</v>
       </c>
       <c r="B786" s="11" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="C786" s="6"/>
       <c r="D786" s="8"/>
@@ -11257,7 +11318,7 @@
         <v>579</v>
       </c>
       <c r="B787" s="11" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="C787" s="6"/>
       <c r="D787" s="8"/>
@@ -11268,7 +11329,7 @@
         <v>579</v>
       </c>
       <c r="B788" s="11" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C788" s="6"/>
       <c r="D788" s="8"/>
@@ -11279,7 +11340,7 @@
         <v>579</v>
       </c>
       <c r="B789" s="11" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C789" s="6"/>
       <c r="D789" s="8"/>
@@ -11290,7 +11351,7 @@
         <v>579</v>
       </c>
       <c r="B790" s="11" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="C790" s="6"/>
       <c r="D790" s="8"/>
@@ -11301,7 +11362,7 @@
         <v>579</v>
       </c>
       <c r="B791" s="11" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="C791" s="6"/>
       <c r="D791" s="8"/>
@@ -11312,7 +11373,7 @@
         <v>579</v>
       </c>
       <c r="B792" s="11" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C792" s="6"/>
       <c r="D792" s="8"/>
@@ -11323,7 +11384,7 @@
         <v>579</v>
       </c>
       <c r="B793" s="11" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C793" s="6"/>
       <c r="D793" s="8"/>
@@ -11334,7 +11395,7 @@
         <v>579</v>
       </c>
       <c r="B794" s="11" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C794" s="6"/>
       <c r="D794" s="8"/>
@@ -11345,7 +11406,7 @@
         <v>579</v>
       </c>
       <c r="B795" s="11" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="C795" s="6"/>
       <c r="D795" s="8"/>
@@ -11356,7 +11417,7 @@
         <v>579</v>
       </c>
       <c r="B796" s="11" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C796" s="6"/>
       <c r="D796" s="8"/>
@@ -11367,7 +11428,7 @@
         <v>579</v>
       </c>
       <c r="B797" s="11" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="C797" s="6"/>
       <c r="D797" s="8"/>
@@ -11378,7 +11439,7 @@
         <v>579</v>
       </c>
       <c r="B798" s="11" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="C798" s="6"/>
       <c r="D798" s="8"/>
@@ -11389,7 +11450,7 @@
         <v>579</v>
       </c>
       <c r="B799" s="11" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="C799" s="6"/>
       <c r="D799" s="8"/>
@@ -11400,7 +11461,7 @@
         <v>579</v>
       </c>
       <c r="B800" s="11" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="C800" s="6"/>
       <c r="D800" s="8"/>
@@ -11411,7 +11472,7 @@
         <v>579</v>
       </c>
       <c r="B801" s="11" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="C801" s="6"/>
       <c r="D801" s="8"/>
@@ -11422,7 +11483,7 @@
         <v>579</v>
       </c>
       <c r="B802" s="11" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="C802" s="6"/>
       <c r="D802" s="8"/>
@@ -11433,7 +11494,7 @@
         <v>579</v>
       </c>
       <c r="B803" s="11" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C803" s="6"/>
       <c r="D803" s="8"/>
@@ -11444,7 +11505,7 @@
         <v>579</v>
       </c>
       <c r="B804" s="11" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C804" s="6"/>
       <c r="D804" s="8"/>
@@ -11455,7 +11516,7 @@
         <v>579</v>
       </c>
       <c r="B805" s="11" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="C805" s="6"/>
       <c r="D805" s="8"/>
@@ -11466,7 +11527,7 @@
         <v>579</v>
       </c>
       <c r="B806" s="11" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="C806" s="6"/>
       <c r="D806" s="8"/>
@@ -11477,7 +11538,7 @@
         <v>579</v>
       </c>
       <c r="B807" s="11" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="C807" s="6"/>
       <c r="D807" s="8"/>
@@ -11488,7 +11549,7 @@
         <v>579</v>
       </c>
       <c r="B808" s="11" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="C808" s="6"/>
       <c r="D808" s="8"/>
@@ -11499,7 +11560,7 @@
         <v>579</v>
       </c>
       <c r="B809" s="11" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="C809" s="6"/>
       <c r="D809" s="8"/>
@@ -11510,7 +11571,7 @@
         <v>579</v>
       </c>
       <c r="B810" s="11" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="C810" s="6"/>
       <c r="D810" s="8"/>
@@ -11521,7 +11582,7 @@
         <v>579</v>
       </c>
       <c r="B811" s="11" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="C811" s="6"/>
       <c r="D811" s="8"/>
@@ -11532,7 +11593,7 @@
         <v>579</v>
       </c>
       <c r="B812" s="11" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="C812" s="6"/>
       <c r="D812" s="8"/>
@@ -11543,7 +11604,7 @@
         <v>579</v>
       </c>
       <c r="B813" s="11" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="C813" s="6"/>
       <c r="D813" s="8"/>
@@ -11554,7 +11615,7 @@
         <v>579</v>
       </c>
       <c r="B814" s="11" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="C814" s="6"/>
       <c r="D814" s="8"/>
@@ -11565,7 +11626,7 @@
         <v>579</v>
       </c>
       <c r="B815" s="11" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="C815" s="6"/>
       <c r="D815" s="8"/>
@@ -11576,7 +11637,7 @@
         <v>579</v>
       </c>
       <c r="B816" s="11" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="C816" s="6"/>
       <c r="D816" s="8"/>
@@ -11587,7 +11648,7 @@
         <v>579</v>
       </c>
       <c r="B817" s="11" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C817" s="6"/>
       <c r="D817" s="8"/>
@@ -11598,7 +11659,7 @@
         <v>579</v>
       </c>
       <c r="B818" s="11" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="C818" s="6"/>
       <c r="D818" s="8"/>
@@ -11609,7 +11670,7 @@
         <v>579</v>
       </c>
       <c r="B819" s="11" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C819" s="6"/>
       <c r="D819" s="8"/>
@@ -11620,7 +11681,7 @@
         <v>579</v>
       </c>
       <c r="B820" s="11" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="C820" s="6"/>
       <c r="D820" s="8"/>
@@ -11631,7 +11692,7 @@
         <v>579</v>
       </c>
       <c r="B821" s="11" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="C821" s="6"/>
       <c r="D821" s="8"/>
@@ -11642,7 +11703,7 @@
         <v>579</v>
       </c>
       <c r="B822" s="11" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="C822" s="6"/>
       <c r="D822" s="8"/>
@@ -11653,7 +11714,7 @@
         <v>579</v>
       </c>
       <c r="B823" s="11" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="C823" s="6"/>
       <c r="D823" s="8"/>
@@ -11664,7 +11725,7 @@
         <v>579</v>
       </c>
       <c r="B824" s="11" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="C824" s="6"/>
       <c r="D824" s="8"/>
@@ -11675,7 +11736,7 @@
         <v>579</v>
       </c>
       <c r="B825" s="11" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="C825" s="6"/>
       <c r="D825" s="8"/>
@@ -11686,7 +11747,7 @@
         <v>579</v>
       </c>
       <c r="B826" s="11" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="C826" s="6"/>
       <c r="D826" s="8"/>
@@ -11697,7 +11758,7 @@
         <v>579</v>
       </c>
       <c r="B827" s="11" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="C827" s="6"/>
       <c r="D827" s="8"/>
@@ -11708,7 +11769,7 @@
         <v>579</v>
       </c>
       <c r="B828" s="11" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C828" s="6"/>
       <c r="D828" s="8"/>
@@ -11719,7 +11780,7 @@
         <v>579</v>
       </c>
       <c r="B829" s="11" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="C829" s="6"/>
       <c r="D829" s="8"/>
@@ -11730,7 +11791,7 @@
         <v>579</v>
       </c>
       <c r="B830" s="11" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="C830" s="6"/>
       <c r="D830" s="8"/>
@@ -11741,7 +11802,7 @@
         <v>579</v>
       </c>
       <c r="B831" s="11" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="C831" s="6"/>
       <c r="D831" s="8"/>
@@ -11752,7 +11813,7 @@
         <v>579</v>
       </c>
       <c r="B832" s="11" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="C832" s="6"/>
       <c r="D832" s="8"/>
@@ -11763,7 +11824,7 @@
         <v>579</v>
       </c>
       <c r="B833" s="11" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="C833" s="6"/>
       <c r="D833" s="8"/>
@@ -11774,7 +11835,7 @@
         <v>579</v>
       </c>
       <c r="B834" s="11" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="C834" s="6"/>
       <c r="D834" s="8"/>
@@ -11785,7 +11846,7 @@
         <v>579</v>
       </c>
       <c r="B835" s="11" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="C835" s="6"/>
       <c r="D835" s="8"/>
@@ -11796,7 +11857,7 @@
         <v>579</v>
       </c>
       <c r="B836" s="11" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="C836" s="6"/>
       <c r="D836" s="8"/>
@@ -11807,7 +11868,7 @@
         <v>579</v>
       </c>
       <c r="B837" s="11" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="C837" s="6"/>
       <c r="D837" s="8"/>
@@ -11818,7 +11879,7 @@
         <v>579</v>
       </c>
       <c r="B838" s="11" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="C838" s="6"/>
       <c r="D838" s="8"/>
@@ -11829,7 +11890,7 @@
         <v>579</v>
       </c>
       <c r="B839" s="11" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="C839" s="6"/>
       <c r="D839" s="8"/>
@@ -11840,7 +11901,7 @@
         <v>579</v>
       </c>
       <c r="B840" s="11" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="C840" s="6"/>
       <c r="D840" s="8"/>
@@ -11851,7 +11912,7 @@
         <v>579</v>
       </c>
       <c r="B841" s="11" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="C841" s="6"/>
       <c r="D841" s="8"/>
@@ -11862,7 +11923,7 @@
         <v>579</v>
       </c>
       <c r="B842" s="11" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="C842" s="6"/>
       <c r="D842" s="8"/>
@@ -11873,7 +11934,7 @@
         <v>579</v>
       </c>
       <c r="B843" s="11" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="C843" s="6"/>
       <c r="D843" s="8"/>
@@ -11884,7 +11945,7 @@
         <v>579</v>
       </c>
       <c r="B844" s="11" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="C844" s="6"/>
       <c r="D844" s="8"/>
@@ -11895,7 +11956,7 @@
         <v>579</v>
       </c>
       <c r="B845" s="11" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C845" s="6"/>
       <c r="D845" s="8"/>
@@ -11906,7 +11967,7 @@
         <v>579</v>
       </c>
       <c r="B846" s="11" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="C846" s="6"/>
       <c r="D846" s="8"/>
@@ -11917,7 +11978,7 @@
         <v>579</v>
       </c>
       <c r="B847" s="11" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="C847" s="6"/>
       <c r="D847" s="8"/>
@@ -11928,7 +11989,7 @@
         <v>579</v>
       </c>
       <c r="B848" s="11" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="C848" s="6"/>
       <c r="D848" s="8"/>
@@ -11939,7 +12000,7 @@
         <v>579</v>
       </c>
       <c r="B849" s="11" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="C849" s="6"/>
       <c r="D849" s="8"/>
@@ -11950,7 +12011,7 @@
         <v>579</v>
       </c>
       <c r="B850" s="11" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="C850" s="6"/>
       <c r="D850" s="8"/>
@@ -11961,7 +12022,7 @@
         <v>579</v>
       </c>
       <c r="B851" s="11" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="C851" s="6"/>
       <c r="D851" s="8"/>
@@ -11972,7 +12033,7 @@
         <v>579</v>
       </c>
       <c r="B852" s="11" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="C852" s="6"/>
       <c r="D852" s="8"/>
@@ -11983,7 +12044,7 @@
         <v>579</v>
       </c>
       <c r="B853" s="11" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="C853" s="6"/>
       <c r="D853" s="8"/>
@@ -11994,7 +12055,7 @@
         <v>579</v>
       </c>
       <c r="B854" s="11" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="C854" s="6"/>
       <c r="D854" s="8"/>
@@ -12005,7 +12066,7 @@
         <v>579</v>
       </c>
       <c r="B855" s="11" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="C855" s="6"/>
       <c r="D855" s="8"/>
@@ -12016,7 +12077,7 @@
         <v>579</v>
       </c>
       <c r="B856" s="11" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="C856" s="6"/>
       <c r="D856" s="8"/>
@@ -12027,7 +12088,7 @@
         <v>579</v>
       </c>
       <c r="B857" s="11" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="C857" s="6"/>
       <c r="D857" s="8"/>
@@ -12038,7 +12099,7 @@
         <v>579</v>
       </c>
       <c r="B858" s="11" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="C858" s="6"/>
       <c r="D858" s="8"/>
@@ -12049,7 +12110,7 @@
         <v>579</v>
       </c>
       <c r="B859" s="11" t="s">
-        <v>279</v>
+        <v>271</v>
       </c>
       <c r="C859" s="6"/>
       <c r="D859" s="8"/>
@@ -12060,7 +12121,7 @@
         <v>579</v>
       </c>
       <c r="B860" s="11" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="C860" s="6"/>
       <c r="D860" s="8"/>
@@ -12071,7 +12132,7 @@
         <v>579</v>
       </c>
       <c r="B861" s="11" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="C861" s="6"/>
       <c r="D861" s="8"/>
@@ -12082,7 +12143,7 @@
         <v>579</v>
       </c>
       <c r="B862" s="11" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="C862" s="6"/>
       <c r="D862" s="8"/>
@@ -12093,7 +12154,7 @@
         <v>579</v>
       </c>
       <c r="B863" s="11" t="s">
-        <v>283</v>
+        <v>275</v>
       </c>
       <c r="C863" s="6"/>
       <c r="D863" s="8"/>
@@ -12104,7 +12165,7 @@
         <v>579</v>
       </c>
       <c r="B864" s="11" t="s">
-        <v>284</v>
+        <v>276</v>
       </c>
       <c r="C864" s="6"/>
       <c r="D864" s="8"/>
@@ -12115,7 +12176,7 @@
         <v>579</v>
       </c>
       <c r="B865" s="11" t="s">
-        <v>285</v>
+        <v>277</v>
       </c>
       <c r="C865" s="6"/>
       <c r="D865" s="8"/>
@@ -12126,7 +12187,7 @@
         <v>579</v>
       </c>
       <c r="B866" s="11" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="C866" s="6"/>
       <c r="D866" s="8"/>
@@ -12137,7 +12198,7 @@
         <v>579</v>
       </c>
       <c r="B867" s="11" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="C867" s="6"/>
       <c r="D867" s="8"/>
@@ -12148,7 +12209,7 @@
         <v>579</v>
       </c>
       <c r="B868" s="11" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
       <c r="C868" s="6"/>
       <c r="D868" s="8"/>
@@ -12159,7 +12220,7 @@
         <v>579</v>
       </c>
       <c r="B869" s="11" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="C869" s="6"/>
       <c r="D869" s="8"/>
@@ -12170,7 +12231,7 @@
         <v>579</v>
       </c>
       <c r="B870" s="11" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="C870" s="6"/>
       <c r="D870" s="8"/>
@@ -12181,7 +12242,7 @@
         <v>579</v>
       </c>
       <c r="B871" s="11" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="C871" s="6"/>
       <c r="D871" s="8"/>
@@ -12192,7 +12253,7 @@
         <v>579</v>
       </c>
       <c r="B872" s="11" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="C872" s="6"/>
       <c r="D872" s="8"/>
@@ -12203,7 +12264,7 @@
         <v>579</v>
       </c>
       <c r="B873" s="11" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="C873" s="6"/>
       <c r="D873" s="8"/>
@@ -12214,7 +12275,7 @@
         <v>579</v>
       </c>
       <c r="B874" s="11" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="C874" s="6"/>
       <c r="D874" s="8"/>
@@ -12225,7 +12286,7 @@
         <v>579</v>
       </c>
       <c r="B875" s="11" t="s">
-        <v>295</v>
+        <v>287</v>
       </c>
       <c r="C875" s="6"/>
       <c r="D875" s="8"/>
@@ -12236,7 +12297,7 @@
         <v>579</v>
       </c>
       <c r="B876" s="11" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="C876" s="6"/>
       <c r="D876" s="8"/>
@@ -12247,7 +12308,7 @@
         <v>579</v>
       </c>
       <c r="B877" s="11" t="s">
-        <v>297</v>
+        <v>289</v>
       </c>
       <c r="C877" s="6"/>
       <c r="D877" s="8"/>
@@ -12258,7 +12319,7 @@
         <v>579</v>
       </c>
       <c r="B878" s="11" t="s">
-        <v>298</v>
+        <v>290</v>
       </c>
       <c r="C878" s="6"/>
       <c r="D878" s="8"/>
@@ -12269,7 +12330,7 @@
         <v>579</v>
       </c>
       <c r="B879" s="11" t="s">
-        <v>299</v>
+        <v>291</v>
       </c>
       <c r="C879" s="6"/>
       <c r="D879" s="8"/>
@@ -12280,7 +12341,7 @@
         <v>579</v>
       </c>
       <c r="B880" s="11" t="s">
-        <v>300</v>
+        <v>292</v>
       </c>
       <c r="C880" s="6"/>
       <c r="D880" s="8"/>
@@ -12291,7 +12352,7 @@
         <v>579</v>
       </c>
       <c r="B881" s="11" t="s">
-        <v>301</v>
+        <v>293</v>
       </c>
       <c r="C881" s="6"/>
       <c r="D881" s="8"/>
@@ -12302,7 +12363,7 @@
         <v>579</v>
       </c>
       <c r="B882" s="11" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="C882" s="6"/>
       <c r="D882" s="8"/>
@@ -12313,7 +12374,7 @@
         <v>579</v>
       </c>
       <c r="B883" s="11" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="C883" s="6"/>
       <c r="D883" s="8"/>
@@ -12324,7 +12385,7 @@
         <v>579</v>
       </c>
       <c r="B884" s="11" t="s">
-        <v>304</v>
+        <v>296</v>
       </c>
       <c r="C884" s="6"/>
       <c r="D884" s="8"/>
@@ -12335,7 +12396,7 @@
         <v>579</v>
       </c>
       <c r="B885" s="11" t="s">
-        <v>305</v>
+        <v>297</v>
       </c>
       <c r="C885" s="6"/>
       <c r="D885" s="8"/>
@@ -12346,7 +12407,7 @@
         <v>579</v>
       </c>
       <c r="B886" s="11" t="s">
-        <v>306</v>
+        <v>298</v>
       </c>
       <c r="C886" s="6"/>
       <c r="D886" s="8"/>
@@ -12357,7 +12418,7 @@
         <v>579</v>
       </c>
       <c r="B887" s="11" t="s">
-        <v>307</v>
+        <v>299</v>
       </c>
       <c r="C887" s="6"/>
       <c r="D887" s="8"/>
@@ -12368,7 +12429,7 @@
         <v>579</v>
       </c>
       <c r="B888" s="11" t="s">
-        <v>308</v>
+        <v>300</v>
       </c>
       <c r="C888" s="6"/>
       <c r="D888" s="8"/>
@@ -12379,7 +12440,7 @@
         <v>579</v>
       </c>
       <c r="B889" s="11" t="s">
-        <v>309</v>
+        <v>301</v>
       </c>
       <c r="C889" s="6"/>
       <c r="D889" s="8"/>
@@ -12390,7 +12451,7 @@
         <v>579</v>
       </c>
       <c r="B890" s="11" t="s">
-        <v>310</v>
+        <v>302</v>
       </c>
       <c r="C890" s="6"/>
       <c r="D890" s="8"/>
@@ -12401,7 +12462,7 @@
         <v>579</v>
       </c>
       <c r="B891" s="11" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="C891" s="6"/>
       <c r="D891" s="8"/>
@@ -12412,7 +12473,7 @@
         <v>579</v>
       </c>
       <c r="B892" s="11" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="C892" s="6"/>
       <c r="D892" s="8"/>
@@ -12423,7 +12484,7 @@
         <v>579</v>
       </c>
       <c r="B893" s="11" t="s">
-        <v>313</v>
+        <v>305</v>
       </c>
       <c r="C893" s="6"/>
       <c r="D893" s="8"/>
@@ -12434,7 +12495,7 @@
         <v>579</v>
       </c>
       <c r="B894" s="11" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="C894" s="6"/>
       <c r="D894" s="8"/>
@@ -12445,7 +12506,7 @@
         <v>579</v>
       </c>
       <c r="B895" s="11" t="s">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="C895" s="6"/>
       <c r="D895" s="8"/>
@@ -12456,7 +12517,7 @@
         <v>579</v>
       </c>
       <c r="B896" s="11" t="s">
-        <v>316</v>
+        <v>308</v>
       </c>
       <c r="C896" s="6"/>
       <c r="D896" s="8"/>
@@ -12467,7 +12528,7 @@
         <v>579</v>
       </c>
       <c r="B897" s="11" t="s">
-        <v>317</v>
+        <v>309</v>
       </c>
       <c r="C897" s="6"/>
       <c r="D897" s="8"/>
@@ -12478,7 +12539,7 @@
         <v>579</v>
       </c>
       <c r="B898" s="11" t="s">
-        <v>318</v>
+        <v>310</v>
       </c>
       <c r="C898" s="6"/>
       <c r="D898" s="8"/>
@@ -12489,7 +12550,7 @@
         <v>579</v>
       </c>
       <c r="B899" s="11" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="C899" s="6"/>
       <c r="D899" s="8"/>
@@ -12500,7 +12561,7 @@
         <v>579</v>
       </c>
       <c r="B900" s="11" t="s">
-        <v>320</v>
+        <v>312</v>
       </c>
       <c r="C900" s="6"/>
       <c r="D900" s="8"/>
@@ -12511,7 +12572,7 @@
         <v>579</v>
       </c>
       <c r="B901" s="11" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="C901" s="6"/>
       <c r="D901" s="8"/>
@@ -12522,7 +12583,7 @@
         <v>579</v>
       </c>
       <c r="B902" s="11" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="C902" s="6"/>
       <c r="D902" s="8"/>
@@ -12533,7 +12594,7 @@
         <v>579</v>
       </c>
       <c r="B903" s="11" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
       <c r="C903" s="6"/>
       <c r="D903" s="8"/>
@@ -12544,7 +12605,7 @@
         <v>579</v>
       </c>
       <c r="B904" s="11" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="C904" s="6"/>
       <c r="D904" s="8"/>
@@ -12555,7 +12616,7 @@
         <v>579</v>
       </c>
       <c r="B905" s="11" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="C905" s="6"/>
       <c r="D905" s="8"/>
@@ -12566,7 +12627,7 @@
         <v>579</v>
       </c>
       <c r="B906" s="11" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="C906" s="6"/>
       <c r="D906" s="8"/>
@@ -12577,7 +12638,7 @@
         <v>579</v>
       </c>
       <c r="B907" s="11" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="C907" s="6"/>
       <c r="D907" s="8"/>
@@ -12588,7 +12649,7 @@
         <v>579</v>
       </c>
       <c r="B908" s="11" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="C908" s="6"/>
       <c r="D908" s="8"/>
@@ -12599,7 +12660,7 @@
         <v>579</v>
       </c>
       <c r="B909" s="11" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="C909" s="6"/>
       <c r="D909" s="8"/>
@@ -12610,7 +12671,7 @@
         <v>579</v>
       </c>
       <c r="B910" s="11" t="s">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="C910" s="6"/>
       <c r="D910" s="8"/>
@@ -12621,7 +12682,7 @@
         <v>579</v>
       </c>
       <c r="B911" s="11" t="s">
-        <v>331</v>
+        <v>323</v>
       </c>
       <c r="C911" s="6"/>
       <c r="D911" s="8"/>
@@ -12632,7 +12693,7 @@
         <v>579</v>
       </c>
       <c r="B912" s="11" t="s">
-        <v>332</v>
+        <v>324</v>
       </c>
       <c r="C912" s="6"/>
       <c r="D912" s="8"/>
@@ -12643,7 +12704,7 @@
         <v>579</v>
       </c>
       <c r="B913" s="11" t="s">
-        <v>333</v>
+        <v>325</v>
       </c>
       <c r="C913" s="6"/>
       <c r="D913" s="8"/>
@@ -12654,7 +12715,7 @@
         <v>579</v>
       </c>
       <c r="B914" s="11" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="C914" s="6"/>
       <c r="D914" s="8"/>
@@ -12665,7 +12726,7 @@
         <v>579</v>
       </c>
       <c r="B915" s="11" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="C915" s="6"/>
       <c r="D915" s="8"/>
@@ -12676,7 +12737,7 @@
         <v>579</v>
       </c>
       <c r="B916" s="11" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="C916" s="6"/>
       <c r="D916" s="8"/>
@@ -12687,7 +12748,7 @@
         <v>579</v>
       </c>
       <c r="B917" s="11" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="C917" s="6"/>
       <c r="D917" s="8"/>
@@ -12698,7 +12759,7 @@
         <v>579</v>
       </c>
       <c r="B918" s="11" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="C918" s="6"/>
       <c r="D918" s="8"/>
@@ -12709,7 +12770,7 @@
         <v>579</v>
       </c>
       <c r="B919" s="11" t="s">
-        <v>339</v>
+        <v>331</v>
       </c>
       <c r="C919" s="6"/>
       <c r="D919" s="8"/>
@@ -12720,7 +12781,7 @@
         <v>579</v>
       </c>
       <c r="B920" s="11" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="C920" s="6"/>
       <c r="D920" s="8"/>
@@ -12731,7 +12792,7 @@
         <v>579</v>
       </c>
       <c r="B921" s="11" t="s">
-        <v>341</v>
+        <v>333</v>
       </c>
       <c r="C921" s="6"/>
       <c r="D921" s="8"/>
@@ -12742,7 +12803,7 @@
         <v>579</v>
       </c>
       <c r="B922" s="11" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="C922" s="6"/>
       <c r="D922" s="8"/>
@@ -12753,7 +12814,7 @@
         <v>579</v>
       </c>
       <c r="B923" s="11" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="C923" s="6"/>
       <c r="D923" s="8"/>
@@ -12764,7 +12825,7 @@
         <v>579</v>
       </c>
       <c r="B924" s="11" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="C924" s="6"/>
       <c r="D924" s="8"/>
@@ -12775,7 +12836,7 @@
         <v>579</v>
       </c>
       <c r="B925" s="11" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="C925" s="6"/>
       <c r="D925" s="8"/>
@@ -12786,7 +12847,7 @@
         <v>579</v>
       </c>
       <c r="B926" s="11" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="C926" s="6"/>
       <c r="D926" s="8"/>
@@ -12797,7 +12858,7 @@
         <v>579</v>
       </c>
       <c r="B927" s="11" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="C927" s="6"/>
       <c r="D927" s="8"/>
@@ -12808,7 +12869,7 @@
         <v>579</v>
       </c>
       <c r="B928" s="11" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="C928" s="6"/>
       <c r="D928" s="8"/>
@@ -12819,7 +12880,7 @@
         <v>579</v>
       </c>
       <c r="B929" s="11" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="C929" s="6"/>
       <c r="D929" s="8"/>
@@ -12830,7 +12891,7 @@
         <v>579</v>
       </c>
       <c r="B930" s="11" t="s">
-        <v>350</v>
+        <v>342</v>
       </c>
       <c r="C930" s="6"/>
       <c r="D930" s="8"/>
@@ -12841,7 +12902,7 @@
         <v>579</v>
       </c>
       <c r="B931" s="11" t="s">
-        <v>351</v>
+        <v>343</v>
       </c>
       <c r="C931" s="6"/>
       <c r="D931" s="8"/>
@@ -12852,7 +12913,7 @@
         <v>579</v>
       </c>
       <c r="B932" s="11" t="s">
-        <v>352</v>
+        <v>344</v>
       </c>
       <c r="C932" s="6"/>
       <c r="D932" s="8"/>
@@ -12863,7 +12924,7 @@
         <v>579</v>
       </c>
       <c r="B933" s="11" t="s">
-        <v>353</v>
+        <v>345</v>
       </c>
       <c r="C933" s="6"/>
       <c r="D933" s="8"/>
@@ -12874,7 +12935,7 @@
         <v>579</v>
       </c>
       <c r="B934" s="11" t="s">
-        <v>354</v>
+        <v>346</v>
       </c>
       <c r="C934" s="6"/>
       <c r="D934" s="8"/>
@@ -12885,7 +12946,7 @@
         <v>579</v>
       </c>
       <c r="B935" s="11" t="s">
-        <v>355</v>
+        <v>347</v>
       </c>
       <c r="C935" s="6"/>
       <c r="D935" s="8"/>
@@ -12896,7 +12957,7 @@
         <v>579</v>
       </c>
       <c r="B936" s="11" t="s">
-        <v>356</v>
+        <v>348</v>
       </c>
       <c r="C936" s="6"/>
       <c r="D936" s="8"/>
@@ -12907,7 +12968,7 @@
         <v>579</v>
       </c>
       <c r="B937" s="11" t="s">
-        <v>357</v>
+        <v>349</v>
       </c>
       <c r="C937" s="6"/>
       <c r="D937" s="8"/>
@@ -12918,7 +12979,7 @@
         <v>579</v>
       </c>
       <c r="B938" s="11" t="s">
-        <v>358</v>
+        <v>350</v>
       </c>
       <c r="C938" s="6"/>
       <c r="D938" s="8"/>
@@ -12929,7 +12990,7 @@
         <v>579</v>
       </c>
       <c r="B939" s="11" t="s">
-        <v>359</v>
+        <v>351</v>
       </c>
       <c r="C939" s="6"/>
       <c r="D939" s="8"/>
@@ -12940,7 +13001,7 @@
         <v>579</v>
       </c>
       <c r="B940" s="11" t="s">
-        <v>360</v>
+        <v>352</v>
       </c>
       <c r="C940" s="6"/>
       <c r="D940" s="8"/>
@@ -12951,7 +13012,7 @@
         <v>579</v>
       </c>
       <c r="B941" s="11" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="C941" s="6"/>
       <c r="D941" s="8"/>
@@ -12962,7 +13023,7 @@
         <v>579</v>
       </c>
       <c r="B942" s="11" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="C942" s="6"/>
       <c r="D942" s="8"/>
@@ -12973,7 +13034,7 @@
         <v>579</v>
       </c>
       <c r="B943" s="11" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="C943" s="6"/>
       <c r="D943" s="8"/>
@@ -12984,7 +13045,7 @@
         <v>579</v>
       </c>
       <c r="B944" s="11" t="s">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="C944" s="6"/>
       <c r="D944" s="8"/>
@@ -12995,72 +13056,104 @@
         <v>579</v>
       </c>
       <c r="B945" s="11" t="s">
-        <v>365</v>
+        <v>357</v>
       </c>
       <c r="C945" s="6"/>
       <c r="D945" s="8"/>
       <c r="E945" s="6"/>
     </row>
-    <row r="946" spans="1:5" ht="14.5" customHeight="1"/>
-    <row r="947" spans="1:5" ht="14.5" customHeight="1"/>
-    <row r="948" spans="1:5" ht="14.5" customHeight="1"/>
-    <row r="949" spans="1:5" ht="14.5" customHeight="1"/>
+    <row r="946" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A946" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B946" s="11" t="s">
+        <v>358</v>
+      </c>
+      <c r="C946" s="6"/>
+      <c r="D946" s="8"/>
+      <c r="E946" s="6"/>
+    </row>
+    <row r="947" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A947" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B947" s="11" t="s">
+        <v>359</v>
+      </c>
+      <c r="C947" s="6"/>
+      <c r="D947" s="8"/>
+      <c r="E947" s="6"/>
+    </row>
+    <row r="948" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A948" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B948" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="C948" s="6"/>
+      <c r="D948" s="8"/>
+      <c r="E948" s="6"/>
+    </row>
+    <row r="949" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A949" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B949" s="11" t="s">
+        <v>361</v>
+      </c>
+      <c r="C949" s="6"/>
+      <c r="D949" s="8"/>
+      <c r="E949" s="6"/>
+    </row>
     <row r="950" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A950" s="6"/>
-      <c r="B950" s="6"/>
+      <c r="A950" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B950" s="11" t="s">
+        <v>362</v>
+      </c>
       <c r="C950" s="6"/>
       <c r="D950" s="8"/>
       <c r="E950" s="6"/>
     </row>
     <row r="951" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A951" s="6"/>
-      <c r="B951" s="6"/>
+      <c r="A951" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B951" s="11" t="s">
+        <v>363</v>
+      </c>
       <c r="C951" s="6"/>
       <c r="D951" s="8"/>
       <c r="E951" s="6"/>
     </row>
     <row r="952" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A952" s="6"/>
-      <c r="B952" s="6"/>
+      <c r="A952" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B952" s="11" t="s">
+        <v>364</v>
+      </c>
       <c r="C952" s="6"/>
       <c r="D952" s="8"/>
       <c r="E952" s="6"/>
     </row>
     <row r="953" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A953" s="6"/>
-      <c r="B953" s="6"/>
+      <c r="A953" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="B953" s="11" t="s">
+        <v>365</v>
+      </c>
       <c r="C953" s="6"/>
       <c r="D953" s="8"/>
       <c r="E953" s="6"/>
     </row>
-    <row r="954" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A954" s="6"/>
-      <c r="B954" s="6"/>
-      <c r="C954" s="6"/>
-      <c r="D954" s="8"/>
-      <c r="E954" s="6"/>
-    </row>
-    <row r="955" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A955" s="6"/>
-      <c r="B955" s="6"/>
-      <c r="C955" s="6"/>
-      <c r="D955" s="8"/>
-      <c r="E955" s="6"/>
-    </row>
-    <row r="956" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A956" s="6"/>
-      <c r="B956" s="6"/>
-      <c r="C956" s="6"/>
-      <c r="D956" s="8"/>
-      <c r="E956" s="6"/>
-    </row>
-    <row r="957" spans="1:5" ht="14.5" customHeight="1">
-      <c r="A957" s="6"/>
-      <c r="B957" s="6"/>
-      <c r="C957" s="6"/>
-      <c r="D957" s="8"/>
-      <c r="E957" s="6"/>
-    </row>
+    <row r="954" spans="1:5" ht="14.5" customHeight="1"/>
+    <row r="955" spans="1:5" ht="14.5" customHeight="1"/>
+    <row r="956" spans="1:5" ht="14.5" customHeight="1"/>
+    <row r="957" spans="1:5" ht="14.5" customHeight="1"/>
     <row r="958" spans="1:5" ht="14.5" customHeight="1">
       <c r="A958" s="6"/>
       <c r="B958" s="6"/>
@@ -13607,6 +13700,62 @@
       <c r="D1035" s="8"/>
       <c r="E1035" s="6"/>
     </row>
+    <row r="1036" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1036" s="6"/>
+      <c r="B1036" s="6"/>
+      <c r="C1036" s="6"/>
+      <c r="D1036" s="8"/>
+      <c r="E1036" s="6"/>
+    </row>
+    <row r="1037" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1037" s="6"/>
+      <c r="B1037" s="6"/>
+      <c r="C1037" s="6"/>
+      <c r="D1037" s="8"/>
+      <c r="E1037" s="6"/>
+    </row>
+    <row r="1038" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1038" s="6"/>
+      <c r="B1038" s="6"/>
+      <c r="C1038" s="6"/>
+      <c r="D1038" s="8"/>
+      <c r="E1038" s="6"/>
+    </row>
+    <row r="1039" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1039" s="6"/>
+      <c r="B1039" s="6"/>
+      <c r="C1039" s="6"/>
+      <c r="D1039" s="8"/>
+      <c r="E1039" s="6"/>
+    </row>
+    <row r="1040" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1040" s="6"/>
+      <c r="B1040" s="6"/>
+      <c r="C1040" s="6"/>
+      <c r="D1040" s="8"/>
+      <c r="E1040" s="6"/>
+    </row>
+    <row r="1041" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1041" s="6"/>
+      <c r="B1041" s="6"/>
+      <c r="C1041" s="6"/>
+      <c r="D1041" s="8"/>
+      <c r="E1041" s="6"/>
+    </row>
+    <row r="1042" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1042" s="6"/>
+      <c r="B1042" s="6"/>
+      <c r="C1042" s="6"/>
+      <c r="D1042" s="8"/>
+      <c r="E1042" s="6"/>
+    </row>
+    <row r="1043" spans="1:5" ht="14.5" customHeight="1">
+      <c r="A1043" s="6"/>
+      <c r="B1043" s="6"/>
+      <c r="C1043" s="6"/>
+      <c r="D1043" s="8"/>
+      <c r="E1043" s="6"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>